<commit_message>
model: check 15 and 16 descriptions match what they test; C1 level 5 and 5.3(d) cite methodology 11.9a
</commit_message>
<xml_diff>
--- a/model/risk-factor-library.xlsx
+++ b/model/risk-factor-library.xlsx
@@ -460,7 +460,7 @@
     <t xml:space="preserve">Structure including a trust, a foundation, a nominee arrangement, or an entity incorporated outside the United Kingdom anywhere in the ownership chain</t>
   </si>
   <si>
-    <t xml:space="preserve">5.3(d), fired on the whole level; see 5.3(d) and methodology 11.9</t>
+    <t xml:space="preserve">5.3(d), fired on the whole level; see 5.3(d) and methodology 11.9a</t>
   </si>
   <si>
     <t xml:space="preserve">Natural person; no beneficial ownership analysis required</t>
@@ -775,7 +775,7 @@
     <t xml:space="preserve">The customer is a money service business, a trust or company service provider, or a dealer in high-value goods.</t>
   </si>
   <si>
-    <t xml:space="preserve">The ownership structure includes nominee shareholders, bearer shares, or an entity incorporated in a jurisdiction with no accessible beneficial ownership register. Because level 5 of factor C1 covers trusts, nominee arrangements and overseas incorporation together, the recorded level cannot tell those apart; the escalator therefore fires on the whole of C1 level 5. That is deliberately conservative and it is the wrong way round: the fix is to split C1 level 5 so the condition can be evaluated, and that is a library change requiring approval (methodology 11.9).</t>
+    <t xml:space="preserve">The ownership structure includes nominee shareholders, bearer shares, or an entity incorporated in a jurisdiction with no accessible beneficial ownership register. Because level 5 of factor C1 covers trusts, nominee arrangements and overseas incorporation together, the recorded level cannot tell those apart; the escalator therefore fires on the whole of C1 level 5. That is deliberately conservative and it is the wrong way round: the fix is to split C1 level 5 so the condition can be evaluated, and that is a library change requiring approval (methodology 11.9a).</t>
   </si>
   <si>
     <t xml:space="preserve">Screening returns a confirmed adverse media match relating to financial crime, fraud, bribery, corruption or tax evasion.</t>

</xml_diff>